<commit_message>
Plantillas HTML de Resend y borrador de la política de datos
- docs/resend/: HTML de ingreso aceptado, crédito aprobado/rechazado y boleta
  del sorteo, con logo y pie de la cooperativa; el correo del código usa el
  mismo diseño.
- /politica-de-datos: borrador según Ley 1581 con los datos faltantes
  resaltados (P-75 a P-81).
- MONTO del correo de crédito con puntos de miles.
- Avances: pendientes nuevos de la política, P-62 hecho, P-72 en curso.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/avances/Avances_Green_Alliance.xlsx
+++ b/docs/avances/Avances_Green_Alliance.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$4:$J$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pendientes'!$A$4:$J$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Plan'!$A$4:$R$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1495,19 +1495,19 @@
         </is>
       </c>
       <c r="C46" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B46,Pendientes!$G$5:$G$78,"Hecho")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B46,Pendientes!$G$5:$G$85,"Hecho")</f>
         <v/>
       </c>
       <c r="D46" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B46,Pendientes!$G$5:$G$78,"En curso")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B46,Pendientes!$G$5:$G$85,"En curso")</f>
         <v/>
       </c>
       <c r="E46" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B46,Pendientes!$G$5:$G$78,"Pendiente")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B46,Pendientes!$G$5:$G$85,"Pendiente")</f>
         <v/>
       </c>
       <c r="F46" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B46,Pendientes!$G$5:$G$78,"Bloqueado")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B46,Pendientes!$G$5:$G$85,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G46" s="9">
@@ -1522,19 +1522,19 @@
         </is>
       </c>
       <c r="C47" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B47,Pendientes!$G$5:$G$78,"Hecho")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B47,Pendientes!$G$5:$G$85,"Hecho")</f>
         <v/>
       </c>
       <c r="D47" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B47,Pendientes!$G$5:$G$78,"En curso")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B47,Pendientes!$G$5:$G$85,"En curso")</f>
         <v/>
       </c>
       <c r="E47" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B47,Pendientes!$G$5:$G$78,"Pendiente")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B47,Pendientes!$G$5:$G$85,"Pendiente")</f>
         <v/>
       </c>
       <c r="F47" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B47,Pendientes!$G$5:$G$78,"Bloqueado")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B47,Pendientes!$G$5:$G$85,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G47" s="9">
@@ -1549,19 +1549,19 @@
         </is>
       </c>
       <c r="C48" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B48,Pendientes!$G$5:$G$78,"Hecho")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B48,Pendientes!$G$5:$G$85,"Hecho")</f>
         <v/>
       </c>
       <c r="D48" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B48,Pendientes!$G$5:$G$78,"En curso")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B48,Pendientes!$G$5:$G$85,"En curso")</f>
         <v/>
       </c>
       <c r="E48" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B48,Pendientes!$G$5:$G$78,"Pendiente")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B48,Pendientes!$G$5:$G$85,"Pendiente")</f>
         <v/>
       </c>
       <c r="F48" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B48,Pendientes!$G$5:$G$78,"Bloqueado")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B48,Pendientes!$G$5:$G$85,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G48" s="9">
@@ -1576,19 +1576,19 @@
         </is>
       </c>
       <c r="C49" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B49,Pendientes!$G$5:$G$78,"Hecho")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B49,Pendientes!$G$5:$G$85,"Hecho")</f>
         <v/>
       </c>
       <c r="D49" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B49,Pendientes!$G$5:$G$78,"En curso")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B49,Pendientes!$G$5:$G$85,"En curso")</f>
         <v/>
       </c>
       <c r="E49" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B49,Pendientes!$G$5:$G$78,"Pendiente")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B49,Pendientes!$G$5:$G$85,"Pendiente")</f>
         <v/>
       </c>
       <c r="F49" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B49,Pendientes!$G$5:$G$78,"Bloqueado")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B49,Pendientes!$G$5:$G$85,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G49" s="9">
@@ -1603,19 +1603,19 @@
         </is>
       </c>
       <c r="C50" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B50,Pendientes!$G$5:$G$78,"Hecho")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B50,Pendientes!$G$5:$G$85,"Hecho")</f>
         <v/>
       </c>
       <c r="D50" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B50,Pendientes!$G$5:$G$78,"En curso")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B50,Pendientes!$G$5:$G$85,"En curso")</f>
         <v/>
       </c>
       <c r="E50" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B50,Pendientes!$G$5:$G$78,"Pendiente")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B50,Pendientes!$G$5:$G$85,"Pendiente")</f>
         <v/>
       </c>
       <c r="F50" s="15">
-        <f>COUNTIFS(Pendientes!$B$5:$B$78,$B50,Pendientes!$G$5:$G$78,"Bloqueado")</f>
+        <f>COUNTIFS(Pendientes!$B$5:$B$85,$B50,Pendientes!$G$5:$G$85,"Bloqueado")</f>
         <v/>
       </c>
       <c r="G50" s="9">
@@ -1639,7 +1639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1774,7 +1774,7 @@
     <row r="6">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>P-43</t>
+          <t>P-72</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1784,17 +1784,17 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Base de datos</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Aplicar en producción la migración 20260923210000_limite_de_intentos.sql</t>
+          <t>Dar a Carlos acceso de colaborador al repo GitHub GreenAllianceCoo/PagGreenAlliance y compartirle el encargo (sin llaves de producción)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Sebas (ga-auditor-supabase revisa antes)</t>
+          <t>Sebas</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
@@ -1804,12 +1804,12 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="21">
@@ -1818,14 +1818,14 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>Crea la tabla limites_intentos y la función registrar_intento, que usan /afiliacion, /ingresar y «Reenviar código» (dentroDelLimite). Sin ella esos límites fallan en producción. Antes del despliegue (6.5). 23-sep: auditada por ga-auditor-supabase, se puede aplicar tal cual (docs/auditorias/2026-09-23-limite-de-intentos.md); falta que Sebas haga db push.</t>
+          <t>Necesario antes de que Carlos pueda abrir PRs a develop desde su propia rama. 24-sep: Sebas ya habló con Carlos para darle el acceso; falta confirmarlo en GitHub.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>P-44</t>
+          <t>P-43</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1835,17 +1835,17 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Variables: SUPABASE_SERVICE_ROLE_KEY, INGRESO_COOKIE_SECRET, LIMITE_HMAC_SECRET, RESEND_API_KEY, EMAIL_FROM, SITIO_URL, RESEND_TEMPLATE_INGRESO_ACEPTADO, RESEND_TEMPLATE_CREDITO_APROBADO, RESEND_TEMPLATE_CREDITO_RECHAZADO, RESEND_TEMPLATE_SORTEO_BOLETA, NEXT_PUBLIC_WHATSAPP</t>
+          <t>Aplicar en producción la migración 20260923210000_limite_de_intentos.sql</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>Sebas (ga-auditor-supabase revisa antes)</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>6.9</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="I7" s="21">
@@ -1869,14 +1869,14 @@
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>NEXT_PUBLIC_WHATSAPP ya tiene dato (P-10, 311 724 1942). LIMITE_HMAC_SECRET: 32+ caracteres, distinto de INGRESO_COOKIE_SECRET, en Production y Preview (sin él el build falla); también en .env.local para `npm start`. 24-sep: SUPABASE_SERVICE_ROLE_KEY da «Invalid API key» en Vercel (P-60) y RESEND_API_KEY, EMAIL_FROM y RESEND_TEMPLATE_SORTEO_BOLETA ahora son obligatorias para el build (P-61).</t>
+          <t>Crea la tabla limites_intentos y la función registrar_intento, que usan /afiliacion, /ingresar y «Reenviar código» (dentroDelLimite). Sin ella esos límites fallan en producción. Antes del despliegue (6.5). 23-sep: auditada por ga-auditor-supabase, se puede aplicar tal cual (docs/auditorias/2026-09-23-limite-de-intentos.md); falta que Sebas haga db push.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>P-45</t>
+          <t>P-44</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1886,17 +1886,17 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Vercel</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Panel de producción: OTP de 6 dígitos, vencimiento del código en 600 s (10 min) e intervalo entre correos ≤ 45 s</t>
+          <t>Variables: SUPABASE_SERVICE_ROLE_KEY, INGRESO_COOKIE_SECRET, LIMITE_HMAC_SECRET, RESEND_API_KEY, EMAIL_FROM, SITIO_URL, RESEND_TEMPLATE_INGRESO_ACEPTADO, RESEND_TEMPLATE_CREDITO_APROBADO, RESEND_TEMPLATE_CREDITO_RECHAZADO, RESEND_TEMPLATE_SORTEO_BOLETA, NEXT_PUBLIC_WHATSAPP</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Yo (panel Supabase/Resend)</t>
+          <t>Yo</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="I8" s="21">
@@ -1920,14 +1920,14 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>Complementa P-19 (SMTP) y P-20 (plantilla Magic Link con {{ .Token }}).</t>
+          <t>NEXT_PUBLIC_WHATSAPP ya tiene dato (P-10, 311 724 1942). LIMITE_HMAC_SECRET: 32+ caracteres, distinto de INGRESO_COOKIE_SECRET, en Production y Preview (sin él el build falla); también en .env.local para `npm start`. 24-sep: SUPABASE_SERVICE_ROLE_KEY da «Invalid API key» en Vercel (P-60) y RESEND_API_KEY, EMAIL_FROM y RESEND_TEMPLATE_SORTEO_BOLETA ahora son obligatorias para el build (P-61). El dominio www.greenallianceco.com ya quedó conectado en Vercel; falta poner SITIO_URL=https://www.greenallianceco.com junto con RESEND_API_KEY, EMAIL_FROM y las 4 RESEND_TEMPLATE_*.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>P-59</t>
+          <t>P-45</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1937,17 +1937,17 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Base de datos</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Aplicar en producción las 9 migraciones de fase 2 (20260924000000…000800) y desplegar enseguida</t>
+          <t>Panel de producción: OTP de 6 dígitos, vencimiento del código en 600 s (10 min) e intervalo entre correos ≤ 45 s</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Sebas (ga-auditor-supabase revisa antes)</t>
+          <t>Yo (panel Supabase/Resend)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>6.13</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="I9" s="21">
@@ -1971,14 +1971,14 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Comprobar que hay 0 afiliaciones en producción antes de hacer db push.</t>
+          <t>Complementa P-19 (SMTP) y P-20 (plantilla Magic Link con {{ .Token }}).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>P-60</t>
+          <t>P-59</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1988,17 +1988,17 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Vercel</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Corregir SUPABASE_SERVICE_ROLE_KEY en Vercel (hoy da «Invalid API key»)</t>
+          <t>Aplicar en producción las 9 migraciones de fase 2 (20260924000000…000800) y desplegar enseguida</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Sebas</t>
+          <t>Sebas (ga-auditor-supabase revisa antes)</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -2013,19 +2013,23 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>6.9</t>
+          <t>6.13</t>
         </is>
       </c>
       <c r="I10" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H10,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J10" s="7" t="inlineStr"/>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>Comprobar que hay 0 afiliaciones en producción antes de hacer db push.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>P-61</t>
+          <t>P-60</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -2035,12 +2039,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Resend</t>
+          <t>Vercel</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Crear en Resend las plantillas de ingreso aceptado, crédito aprobado/rechazado y boleta del sorteo (ga-sorteo-boleta); confirmar el tope de 3 reenvíos de boleta al día</t>
+          <t>Corregir SUPABASE_SERVICE_ROLE_KEY en Vercel (hoy da «Invalid API key»)</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -2067,16 +2071,12 @@
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H11,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>RESEND_API_KEY, EMAIL_FROM y RESEND_TEMPLATE_SORTEO_BOLETA ya son obligatorias para el build.</t>
-        </is>
-      </c>
+      <c r="J11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>P-72</t>
+          <t>P-61</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Resend</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Dar a Carlos acceso de colaborador al repo GitHub GreenAllianceCoo/PagGreenAlliance y compartirle el encargo (sin llaves de producción)</t>
+          <t>Crear en Resend las plantillas de ingreso aceptado, crédito aprobado/rechazado y boleta del sorteo (ga-sorteo-boleta); confirmar el tope de 3 reenvíos de boleta al día</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="I12" s="21">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>Necesario antes de que Carlos pueda abrir PRs a develop desde su propia rama.</t>
+          <t>RESEND_API_KEY, EMAIL_FROM y RESEND_TEMPLATE_SORTEO_BOLETA ya son obligatorias para el build. 24-sep: el HTML de las 4 plantillas (ingreso aceptado, crédito aprobado, crédito rechazado, boleta del sorteo) ya está listo en docs/resend/, con el mismo diseño del correo del código; falta que Sebas las cree y publique en Resend.</t>
         </is>
       </c>
     </row>
@@ -3708,14 +3708,14 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>Ruta /politica-de-datos ya existe (placeholder). 24-sep: debe incluir la autorización de datos sensibles para las fotos de cédula y la selfie (Ley 1581). Bloquea el despliegue.</t>
+          <t>Ruta /politica-de-datos ya existe. 24-sep: borrador completo con 10 secciones (Ley 1581, Decreto 1377) y la autorización de datos sensibles para fotos y selfie; los datos que faltan quedan resaltados en la página con &lt;Pendiente&gt;. Faltan de la cooperativa: NIT/dirección/ciudad (P-75), fecha de vigencia (P-76), país o región de los servidores -Supabase, Vercel, Resend- (P-77), alternativa de verificación sin selfie (P-78), plazos de conservación de fotos y demás datos (P-79, ligado a P-63) y si reportan a centrales de riesgo Ley 1266 (P-80); y falta revisión de un abogado (P-81). Bloquea el despliegue.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>P-13</t>
+          <t>P-75</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -3725,12 +3725,12 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Configuración</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Texto de vigilancia de Supersolidaria (TEXTO_VIGILANCIA)</t>
+          <t>NIT, dirección y ciudad de la cooperativa para la política de datos</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G45" s="8" t="inlineStr">
@@ -3750,19 +3750,23 @@
       </c>
       <c r="H45" s="8" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="I45" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H45,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J45" s="7" t="inlineStr"/>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>24-sep: reportado por la sesión principal, necesario para publicar /politica-de-datos.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="19" t="inlineStr">
         <is>
-          <t>P-46</t>
+          <t>P-76</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3772,12 +3776,12 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>/afiliacion</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Nombres oficiales de los grados</t>
+          <t>Fecha de vigencia de la política de datos</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -3787,7 +3791,7 @@
       </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G46" s="8" t="inlineStr">
@@ -3797,7 +3801,7 @@
       </c>
       <c r="H46" s="8" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="I46" s="21">
@@ -3806,14 +3810,14 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>Se usan en el select «Grado» (grados_credito).</t>
+          <t>24-sep: reportado por la sesión principal.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="19" t="inlineStr">
         <is>
-          <t>P-47</t>
+          <t>P-77</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -3823,12 +3827,12 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>/cuenta</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Estado de desembolso (cómo y cuándo se informa al asociado)</t>
+          <t>País o región de los servidores (Supabase, Vercel, Resend)</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -3838,7 +3842,7 @@
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G47" s="8" t="inlineStr">
@@ -3848,7 +3852,7 @@
       </c>
       <c r="H47" s="8" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="I47" s="21">
@@ -3857,14 +3861,14 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>Reportado por ga-funcionalidad-botones el 23-sep.</t>
+          <t>24-sep: reportado por la sesión principal, dato exigido por la Ley 1581 para informar transferencia internacional de datos.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="19" t="inlineStr">
         <is>
-          <t>P-16</t>
+          <t>P-78</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3874,12 +3878,12 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Landing</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Fotos reales, cifras y testimonios</t>
+          <t>Alternativa de verificación para quien no quiera subir la selfie</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -3889,7 +3893,7 @@
       </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G48" s="8" t="inlineStr">
@@ -3899,7 +3903,7 @@
       </c>
       <c r="H48" s="8" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="I48" s="21">
@@ -3908,14 +3912,14 @@
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
-          <t>23-sep: los espacios de foto de la landing ya tienen diseño de marca (EspacioFoto). Para poner la foto real se cambia `null` por { src, alt }. Faltan las fotos de la cooperativa.</t>
+          <t>24-sep: reportado por la sesión principal.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="19" t="inlineStr">
         <is>
-          <t>P-18</t>
+          <t>P-79</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
@@ -3925,12 +3929,12 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Asociados</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Correos reales de los asociados (Excel de importación)</t>
+          <t>Plazos de conservación de los datos (fotos de rechazados y de asociados, y demás datos)</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -3945,12 +3949,12 @@
       </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H49" s="8" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="I49" s="21">
@@ -3959,14 +3963,14 @@
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>Ya no aplica: decisión de la cooperativa 2026-09-24, no habrá importación de Excel. El ingreso ahora se resuelve con la afiliación v2 (correo institucional propio) más aprobación en /admin.</t>
+          <t>24-sep: reportado por la sesión principal; el plazo de las fotos es el mismo que decida P-63 (borrado automático de fotos rechazadas, 5.10).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="19" t="inlineStr">
         <is>
-          <t>P-10</t>
+          <t>P-13</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3981,7 +3985,7 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Número de WhatsApp (NEXT_PUBLIC_WHATSAPP)</t>
+          <t>Texto de vigilancia de Supersolidaria (TEXTO_VIGILANCIA)</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -3996,7 +4000,7 @@
       </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr">
@@ -4008,16 +4012,12 @@
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H50,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J50" s="7" t="inlineStr">
-        <is>
-          <t>24-sep: 311 724 1942.</t>
-        </is>
-      </c>
+      <c r="J50" s="7" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="19" t="inlineStr">
         <is>
-          <t>P-11</t>
+          <t>P-46</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
@@ -4027,12 +4027,12 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Configuración</t>
+          <t>/afiliacion</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Días hábiles de respuesta (DIAS_RESPUESTA)</t>
+          <t>Nombres oficiales de los grados</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -4047,7 +4047,7 @@
       </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H51" s="8" t="inlineStr">
@@ -4061,14 +4061,14 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>24-sep: la cooperativa dio el tiempo de respuesta como «4 horas o menos» (ver P-17); se usa ese dato en vez de días hábiles.</t>
+          <t>Se usan en el select «Grado» (grados_credito).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="19" t="inlineStr">
         <is>
-          <t>P-12</t>
+          <t>P-47</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -4078,12 +4078,12 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Configuración</t>
+          <t>/cuenta</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Correo de contacto (CORREO_CONTACTO)</t>
+          <t>Estado de desembolso (cómo y cuándo se informa al asociado)</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr">
@@ -4112,14 +4112,14 @@
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>24-sep: soporte@greenallianceco.com.</t>
+          <t>Reportado por ga-funcionalidad-botones el 23-sep.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="19" t="inlineStr">
         <is>
-          <t>P-15</t>
+          <t>P-80</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
@@ -4129,17 +4129,17 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>/cuenta</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Destino de «Nueva solicitud» (nav y acceso rápido)</t>
+          <t>Si van a reportar a centrales de riesgo (Ley 1266, autorización aparte)</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>Cooperativa</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -4149,12 +4149,12 @@
       </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="I53" s="21">
@@ -4163,14 +4163,14 @@
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Hoy es href="#".</t>
+          <t>24-sep: reportado por la sesión principal.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="19" t="inlineStr">
         <is>
-          <t>P-17</t>
+          <t>P-16</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Tiempo de respuesta real ([TIEMPO] y [T])</t>
+          <t>Fotos reales, cifras y testimonios</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr">
@@ -4214,34 +4214,34 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>24-sep: «4 horas o menos».</t>
+          <t>23-sep: los espacios de foto de la landing ya tienen diseño de marca (EspacioFoto). Para poner la foto real se cambia `null` por { src, alt }. Faltan las fotos de la cooperativa.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="19" t="inlineStr">
         <is>
-          <t>P-58</t>
+          <t>P-18</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Verificación y cierre</t>
+          <t>Dato de la cooperativa</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Pruebas</t>
+          <t>Asociados</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Actualizar tests/e2e a la afiliación v2 y a la nueva máscara de correo</t>
+          <t>Correos reales de los asociados (Excel de importación)</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>ga-escritor-tests</t>
+          <t>Cooperativa</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -4251,12 +4251,12 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="I55" s="21">
@@ -4265,128 +4265,136 @@
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>d-afiliacion.spec.ts usa el formulario viejo (nombres y apellidos, unidad) y hace falta reescribirlo entero para institución/Nequi/asesor/fotos (k-roles.spec.ts ya cubre un caso feliz v2 pero no reemplaza la cobertura de D). 24-sep: ga-escritor-tests lo reescribió entero (48 pruebas × 2 proyectos); 92/96 pasan, 4 fallan por un bug real de la app (ver P-74), no de la prueba. b-ingreso.spec.ts, i-despliegue.spec.ts y j-produccion.spec.ts siguen con el formato viejo de máscara de correo y dominios (formato nuevo xx•••@yy•••.co); ese trabajo pasa a Carlos Pardo (ver P-71, 6.15). Falta correr npm run test:db (pgTAP), bloqueado por el permiso de la sandbox. Actualización: el bug de P-74 ya está corregido y d-afiliacion pasa 96/96; pgTAP 222/222 corrido por la sesión principal.</t>
+          <t>Ya no aplica: decisión de la cooperativa 2026-09-24, no habrá importación de Excel. El ingreso ahora se resuelve con la afiliación v2 (correo institucional propio) más aprobación en /admin.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="19" t="inlineStr">
         <is>
-          <t>P-42</t>
+          <t>P-10</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Verificación y cierre</t>
+          <t>Dato de la cooperativa</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Despliegue</t>
+          <t>Configuración</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Subir a GitHub y desplegar en Vercel</t>
+          <t>Número de WhatsApp (NEXT_PUBLIC_WHATSAPP)</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>Cooperativa</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="I56" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H56,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J56" s="7" t="inlineStr"/>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>24-sep: 311 724 1942.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="19" t="inlineStr">
         <is>
-          <t>P-64</t>
+          <t>P-11</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Verificación y cierre</t>
+          <t>Dato de la cooperativa</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Configuración</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Abrir el PR de develop a main</t>
+          <t>Días hábiles de respuesta (DIAS_RESPUESTA)</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Sebas</t>
+          <t>Cooperativa</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="I57" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H57,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J57" s="7" t="inlineStr"/>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>24-sep: la cooperativa dio el tiempo de respuesta como «4 horas o menos» (ver P-17); se usa ese dato en vez de días hábiles.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="19" t="inlineStr">
         <is>
-          <t>P-62</t>
+          <t>P-12</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Verificación y cierre</t>
+          <t>Dato de la cooperativa</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Base de datos</t>
+          <t>Configuración</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Borrar la cuenta admin de prueba «Test QA» (cédula 1099887766) desde el panel de Supabase</t>
+          <t>Correo de contacto (CORREO_CONTACTO)</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>Sebas</t>
+          <t>Cooperativa</t>
         </is>
       </c>
       <c r="F58" s="8" t="inlineStr">
@@ -4396,12 +4404,12 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>6.13</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="I58" s="21">
@@ -4410,34 +4418,34 @@
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>Ya hay 3 administradores reales en producción: Ricardo, Abogados Prieto y Sebas.</t>
+          <t>24-sep: soporte@greenallianceco.com.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="19" t="inlineStr">
         <is>
-          <t>P-70</t>
+          <t>P-15</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Verificación y cierre</t>
+          <t>Dato de la cooperativa</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>QA</t>
+          <t>/cuenta</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Pruebas en celulares reales (Android e iPhone): cámara, código, sorteo, crédito y correos en Gmail/Outlook, con informe y capturas</t>
+          <t>Destino de «Nueva solicitud» (nav y acceso rápido)</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Carlos Pardo</t>
+          <t>Yo</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -4447,12 +4455,12 @@
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>6.14</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="I59" s="21">
@@ -4461,49 +4469,49 @@
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>Encargo externo (500.000 COP) por PR a develop. Ver P-73.</t>
+          <t>Hoy es href="#".</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="19" t="inlineStr">
         <is>
-          <t>P-71</t>
+          <t>P-17</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Verificación y cierre</t>
+          <t>Dato de la cooperativa</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Pruebas</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Actualizar tests/e2e b-ingreso, i-despliegue y j-produccion al formato nuevo de máscara de correo</t>
+          <t>Tiempo de respuesta real ([TIEMPO] y [T])</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>Carlos Pardo</t>
+          <t>Cooperativa</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>6.15</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="I60" s="21">
@@ -4512,14 +4520,14 @@
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>Encargo externo (500.000 COP) por PR a develop. Parte del alcance que P-58 dejó fuera. Ver P-73.</t>
+          <t>24-sep: «4 horas o menos».</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="19" t="inlineStr">
         <is>
-          <t>P-39</t>
+          <t>P-58</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
@@ -4529,17 +4537,17 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Calidad</t>
+          <t>Pruebas</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Correr ga-verificador-qa y ga-verificador-responsive</t>
+          <t>Actualizar tests/e2e a la afiliación v2 y a la nueva máscara de correo</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>ga-escritor-tests</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -4549,12 +4557,12 @@
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="I61" s="21">
@@ -4563,14 +4571,14 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>QA 1 hecha el 23-sep (186 pasan, 2 fallan; informe docs/verificaciones/2026-09-23-verificacion-1.md). Responsive hecha el 23-sep: 2 fallas de scroll corregidas (5.8) y segunda pasada con 0 fallas en 13 anchos (320–1920 px); tests/responsive 10/10. La QA final sigue en 6.3.</t>
+          <t>d-afiliacion.spec.ts usa el formulario viejo (nombres y apellidos, unidad) y hace falta reescribirlo entero para institución/Nequi/asesor/fotos (k-roles.spec.ts ya cubre un caso feliz v2 pero no reemplaza la cobertura de D). 24-sep: ga-escritor-tests lo reescribió entero (48 pruebas × 2 proyectos); 92/96 pasan, 4 fallan por un bug real de la app (ver P-74), no de la prueba. b-ingreso.spec.ts, i-despliegue.spec.ts y j-produccion.spec.ts siguen con el formato viejo de máscara de correo y dominios (formato nuevo xx•••@yy•••.co); ese trabajo pasa a Carlos Pardo (ver P-71, 6.15). Falta correr npm run test:db (pgTAP), bloqueado por el permiso de la sandbox. Actualización: el bug de P-74 ya está corregido y d-afiliacion pasa 96/96; pgTAP 222/222 corrido por la sesión principal.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="19" t="inlineStr">
         <is>
-          <t>P-41</t>
+          <t>P-42</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -4580,12 +4588,12 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Despliegue</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>Commit de las pantallas nuevas</t>
+          <t>Subir a GitHub y desplegar en Vercel</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
@@ -4600,28 +4608,24 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="I62" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H62,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J62" s="7" t="inlineStr">
-        <is>
-          <t>Commit d86db86 en develop.</t>
-        </is>
-      </c>
+      <c r="J62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="19" t="inlineStr">
         <is>
-          <t>P-40</t>
+          <t>P-64</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
@@ -4631,48 +4635,44 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>Código</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Borrar /login y /dashboard cuando /ingresar y /cuenta funcionen</t>
+          <t>Abrir el PR de develop a main</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>Sebas</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="I63" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H63,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J63" s="7" t="inlineStr">
-        <is>
-          <t>Borradas el 23-sep (incluida /dashboard/solicitar, su parte del proxy y los colores heredados de tailwind.config.ts).</t>
-        </is>
-      </c>
+      <c r="J63" s="7" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="19" t="inlineStr">
         <is>
-          <t>P-49</t>
+          <t>P-81</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -4682,32 +4682,32 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Seguridad</t>
+          <t>Legal</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Revisar si conviene confiar en x-forwarded-for para el límite de intentos por IP</t>
+          <t>Revisión de la política de datos por un abogado</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>ga-revisor-seguridad</t>
+          <t>Sebas</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="I64" s="21">
@@ -4716,14 +4716,14 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>Sugerido por ga-verificador-qa el 23-sep. Documentado por ga-funcionalidad-botones como O-01 en lib/servidor/limite.ts: x-forwarded-for/x-real-ip solo son confiables detrás de Vercel (nuestro caso); el límite real por cédula/IP lo hace la app, no Supabase.</t>
+          <t>24-sep: reportado por la sesión principal; falta antes de publicar /politica-de-datos.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="19" t="inlineStr">
         <is>
-          <t>P-50</t>
+          <t>P-70</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
@@ -4733,17 +4733,17 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Correos</t>
+          <t>QA</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Confirmar que salen los correos de afiliación (el log queda en la terminal de next dev)</t>
+          <t>Pruebas en celulares reales (Android e iPhone): cámara, código, sorteo, crédito y correos en Gmail/Outlook, con informe y capturas</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>Carlos Pardo</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -4753,12 +4753,12 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>6.14</t>
         </is>
       </c>
       <c r="I65" s="21">
@@ -4767,14 +4767,14 @@
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>Ya no aplica: el 23-sep se quitaron los correos de afiliación del código (decisión de Sebas).</t>
+          <t>Encargo externo (500.000 COP) por PR a develop. Ver P-73.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="19" t="inlineStr">
         <is>
-          <t>P-52</t>
+          <t>P-71</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -4784,32 +4784,32 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Documentación</t>
+          <t>Pruebas</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>Mapa de botones: §4 «Nueva solicitud» → /cuenta/solicitar y sección para la ruta /cuenta/solicitar</t>
+          <t>Actualizar tests/e2e b-ingreso, i-despliegue y j-produccion al formato nuevo de máscara de correo</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>ga-funcionalidad-botones</t>
+          <t>Carlos Pardo</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>6.15</t>
         </is>
       </c>
       <c r="I66" s="21">
@@ -4818,34 +4818,34 @@
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>Reportado por ga-diseno-a-codigo. Verificado el 23-sep: docs/mapa-de-botones.md ya tiene §4 «Nueva solicitud» → /cuenta/solicitar (Definido) y §4b /cuenta/solicitar; /dashboard se eliminó.</t>
+          <t>Encargo externo (500.000 COP) por PR a develop. Parte del alcance que P-58 dejó fuera. Ver P-73.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="19" t="inlineStr">
         <is>
-          <t>P-63</t>
+          <t>P-39</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Verificación y cierre</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Calidad</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Preguntas abiertas de fase 2 para la cooperativa: grados del Ejército, dominios de correo institucionales (hoy solo policia.gov.co, buzonejercito.mil.co, ejercito.mil.co), tiempo que se guardan las fotos y tope de intentos del sorteo</t>
+          <t>Correr ga-verificador-qa y ga-verificador-responsive</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Cooperativa</t>
+          <t>Yo</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -4855,12 +4855,12 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="I67" s="21">
@@ -4869,49 +4869,49 @@
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>Ver docs/spec-fase-2.md §Preguntas abiertas.</t>
+          <t>QA 1 hecha el 23-sep (186 pasan, 2 fallan; informe docs/verificaciones/2026-09-23-verificacion-1.md). Responsive hecha el 23-sep: 2 fallas de scroll corregidas (5.8) y segunda pasada con 0 fallas en 13 anchos (320–1920 px); tests/responsive 10/10. La QA final sigue en 6.3.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="19" t="inlineStr">
         <is>
-          <t>P-02</t>
+          <t>P-41</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Verificación y cierre</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>/cuenta</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>Preguntar a la cooperativa si los convenios tendrán página propia</t>
+          <t>Commit de las pantallas nuevas</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>Cooperativa</t>
+          <t>Yo</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I68" s="21">
@@ -4920,29 +4920,29 @@
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
-          <t>Por ahora son una sección en /cuenta (#convenios).</t>
+          <t>Commit d86db86 en develop.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="19" t="inlineStr">
         <is>
-          <t>P-53</t>
+          <t>P-40</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Verificación y cierre</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Landing</t>
+          <t>Código</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>A 320 px la línea «COOPERATIVA» del logo mide ~5 px de alto (opcional: ocultarla o achicar «Ingresar» bajo 360 px)</t>
+          <t>Borrar /login y /dashboard cuando /ingresar y /cuenta funcionen</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
@@ -4952,17 +4952,17 @@
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="I69" s="21">
@@ -4971,39 +4971,39 @@
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>Menor y opcional, reportado por ga-verificador-responsive el 23-sep.</t>
+          <t>Borradas el 23-sep (incluida /dashboard/solicitar, su parte del proxy y los colores heredados de tailwind.config.ts).</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="19" t="inlineStr">
         <is>
-          <t>P-09</t>
+          <t>P-49</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Verificación y cierre</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Base de datos</t>
+          <t>Seguridad</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>Revisar y aplicar en producción la migración blindar_solicitudes_y_revisiones</t>
+          <t>Revisar si conviene confiar en x-forwarded-for para el límite de intentos por IP</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>Sebas (ga-auditor-supabase revisa antes)</t>
+          <t>ga-revisor-seguridad</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G70" s="8" t="inlineStr">
@@ -5013,7 +5013,7 @@
       </c>
       <c r="H70" s="8" t="inlineStr">
         <is>
-          <t>6.10</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="I70" s="21">
@@ -5022,29 +5022,29 @@
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>Verificado con list_migrations el 23-sep: producción ya tiene 20260923173355_blindar_solicitudes_y_revisiones.</t>
+          <t>Sugerido por ga-verificador-qa el 23-sep. Documentado por ga-funcionalidad-botones como O-01 en lib/servidor/limite.ts: x-forwarded-for/x-real-ip solo son confiables detrás de Vercel (nuestro caso); el límite real por cédula/IP lo hace la app, no Supabase.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="19" t="inlineStr">
         <is>
-          <t>P-08</t>
+          <t>P-50</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Verificación y cierre</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>/cuenta</t>
+          <t>Correos</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>P-10: el asociado no cambia su nombre pero sí su teléfono</t>
+          <t>Confirmar que salen los correos de afiliación (el log queda en la terminal de next dev)</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="H71" s="8" t="inlineStr">
         <is>
-          <t>3.6</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I71" s="21">
@@ -5073,34 +5073,34 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>Apartado «Mis datos» ya maquetado.</t>
+          <t>Ya no aplica: el 23-sep se quitaron los correos de afiliación del código (decisión de Sebas).</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="19" t="inlineStr">
         <is>
-          <t>P-65</t>
+          <t>P-62</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Verificación y cierre</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Sorteo</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>Decidir si un admin o un asesor pueden participar en el sorteo mensual</t>
+          <t>Borrar la cuenta admin de prueba «Test QA» (cédula 1099887766) desde el panel de Supabase</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>Cooperativa</t>
+          <t>Sebas</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="H72" s="8" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>6.13</t>
         </is>
       </c>
       <c r="I72" s="21">
@@ -5124,34 +5124,34 @@
       </c>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>Sugerido por ga-revisor-seguridad el 24-sep. 24-sep: decidido que solo participan asociados (S-13, ya implementado en participarSorteo).</t>
+          <t>Ya hay 3 administradores reales en producción: Ricardo, Abogados Prieto y Sebas. 24-sep: usuario «Test QA» borrado de producción por Sebas.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="19" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>P-52</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Verificación y cierre</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Documentación</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Color de error #B3261E</t>
+          <t>Mapa de botones: §4 «Nueva solicitud» → /cuenta/solicitar y sección para la ruta /cuenta/solicitar</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>ga-funcionalidad-botones</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="H73" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3.7</t>
         </is>
       </c>
       <c r="I73" s="21">
@@ -5175,14 +5175,14 @@
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>Se deja.</t>
+          <t>Reportado por ga-diseno-a-codigo. Verificado el 23-sep: docs/mapa-de-botones.md ya tiene §4 «Nueva solicitud» → /cuenta/solicitar (Definido) y §4b /cuenta/solicitar; /dashboard se eliminó.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="19" t="inlineStr">
         <is>
-          <t>P-03</t>
+          <t>P-63</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -5192,32 +5192,32 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>/cuenta</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>Estado vacío de «Tu solicitud»</t>
+          <t>Preguntas abiertas de fase 2 para la cooperativa: grados del Ejército, dominios de correo institucionales (hoy solo policia.gov.co, buzonejercito.mil.co, ejercito.mil.co), tiempo que se guardan las fotos y tope de intentos del sorteo</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>Cooperativa</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H74" s="8" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="I74" s="21">
@@ -5226,14 +5226,14 @@
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>Ver con /cuenta?vacio=1.</t>
+          <t>Ver docs/spec-fase-2.md §Preguntas abiertas.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="19" t="inlineStr">
         <is>
-          <t>P-04</t>
+          <t>P-02</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
@@ -5243,17 +5243,17 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>/cuenta</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>Logo en celular como enlace a la landing</t>
+          <t>Preguntar a la cooperativa si los convenios tendrán página propia</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>Cooperativa</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
@@ -5263,24 +5263,28 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H75" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="I75" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H75,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J75" s="7" t="inlineStr"/>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>Por ahora son una sección en /cuenta (#convenios).</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="19" t="inlineStr">
         <is>
-          <t>P-05</t>
+          <t>P-53</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
@@ -5290,12 +5294,12 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Landing</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>Escudo: public/logos/vector/green-alliance-logo.svg</t>
+          <t>A 320 px la línea «COOPERATIVA» del logo mide ~5 px de alto (opcional: ocultarla o achicar «Ingresar» bajo 360 px)</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -5310,7 +5314,7 @@
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="H76" s="8" t="inlineStr">
@@ -5322,12 +5326,16 @@
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H76,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J76" s="7" t="inlineStr"/>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>Menor y opcional, reportado por ga-verificador-responsive el 23-sep.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="19" t="inlineStr">
         <is>
-          <t>P-06</t>
+          <t>P-09</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
@@ -5337,22 +5345,22 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>/ingresar</t>
+          <t>Base de datos</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>Formulario de ingreso entre 640 y 767 px (columna de 440 px)</t>
+          <t>Revisar y aplicar en producción la migración blindar_solicitudes_y_revisiones</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>Yo</t>
+          <t>Sebas (ga-auditor-supabase revisa antes)</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G77" s="8" t="inlineStr">
@@ -5362,19 +5370,23 @@
       </c>
       <c r="H77" s="8" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>6.10</t>
         </is>
       </c>
       <c r="I77" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H77,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J77" s="7" t="inlineStr"/>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>Verificado con list_migrations el 23-sep: producción ya tiene 20260923173355_blindar_solicitudes_y_revisiones.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="19" t="inlineStr">
         <is>
-          <t>P-07</t>
+          <t>P-08</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
@@ -5384,12 +5396,12 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>/ingresar</t>
+          <t>/cuenta</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>Panel verde en tableta (640–1023 px) centrado</t>
+          <t>P-10: el asociado no cambia su nombre pero sí su teléfono</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
@@ -5399,7 +5411,7 @@
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G78" s="8" t="inlineStr">
@@ -5409,18 +5421,363 @@
       </c>
       <c r="H78" s="8" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>3.6</t>
         </is>
       </c>
       <c r="I78" s="21">
         <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H78,Plan!$A$5:$A$64,0)),"—")</f>
         <v/>
       </c>
-      <c r="J78" s="7" t="inlineStr"/>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>Apartado «Mis datos» ya maquetado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="19" t="inlineStr">
+        <is>
+          <t>P-65</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Sorteo</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>Decidir si un admin o un asesor pueden participar en el sorteo mensual</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Cooperativa</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H79" s="8" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="I79" s="21">
+        <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H79,Plan!$A$5:$A$64,0)),"—")</f>
+        <v/>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>Sugerido por ga-revisor-seguridad el 24-sep. 24-sep: decidido que solo participan asociados (S-13, ya implementado en participarSorteo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="19" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Color de error #B3261E</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Yo</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G80" s="8" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H80" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I80" s="21">
+        <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H80,Plan!$A$5:$A$64,0)),"—")</f>
+        <v/>
+      </c>
+      <c r="J80" s="7" t="inlineStr">
+        <is>
+          <t>Se deja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="19" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>/cuenta</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Estado vacío de «Tu solicitud»</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Yo</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H81" s="8" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="I81" s="21">
+        <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H81,Plan!$A$5:$A$64,0)),"—")</f>
+        <v/>
+      </c>
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>Ver con /cuenta?vacio=1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="19" t="inlineStr">
+        <is>
+          <t>P-04</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Logo en celular como enlace a la landing</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>Yo</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I82" s="21">
+        <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H82,Plan!$A$5:$A$64,0)),"—")</f>
+        <v/>
+      </c>
+      <c r="J82" s="7" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="19" t="inlineStr">
+        <is>
+          <t>P-05</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Escudo: public/logos/vector/green-alliance-logo.svg</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>Yo</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G83" s="8" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H83" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I83" s="21">
+        <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H83,Plan!$A$5:$A$64,0)),"—")</f>
+        <v/>
+      </c>
+      <c r="J83" s="7" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="19" t="inlineStr">
+        <is>
+          <t>P-06</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>/ingresar</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr">
+        <is>
+          <t>Formulario de ingreso entre 640 y 767 px (columna de 440 px)</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>Yo</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="I84" s="21">
+        <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H84,Plan!$A$5:$A$64,0)),"—")</f>
+        <v/>
+      </c>
+      <c r="J84" s="7" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="19" t="inlineStr">
+        <is>
+          <t>P-07</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>/ingresar</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Panel verde en tableta (640–1023 px) centrado</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>Yo</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="H85" s="8" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="I85" s="21">
+        <f>IFERROR(INDEX(Plan!$B$5:$B$64,MATCH(H85,Plan!$A$5:$A$64,0)),"—")</f>
+        <v/>
+      </c>
+      <c r="J85" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J78"/>
-  <conditionalFormatting sqref="G5:G78">
+  <autoFilter ref="A4:J85"/>
+  <conditionalFormatting sqref="G5:G85">
     <cfRule type="expression" priority="1" dxfId="1">
       <formula>$G5="Hecho"</formula>
     </cfRule>
@@ -5434,7 +5791,7 @@
       <formula>$G5="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5:F78">
+  <conditionalFormatting sqref="F5:F85">
     <cfRule type="expression" priority="5" dxfId="5">
       <formula>$F5="Alta"</formula>
     </cfRule>
@@ -5445,16 +5802,16 @@
       <formula>$F5="Baja"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:F78">
+  <conditionalFormatting sqref="A5:F85">
     <cfRule type="expression" priority="8" dxfId="8">
       <formula>$G5="Hecho"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="G5:G78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G5:G85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Hecho,En curso,Pendiente,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Alta,Media,Baja"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8647,7 +9004,7 @@
       </c>
       <c r="R43" s="7" t="inlineStr">
         <is>
-          <t>Página placeholder lista; falta el texto de la política, incluida la autorización de datos sensibles para las fotos de cédula y la selfie (Ley 1581). Bloquea el despliegue (6.5).</t>
+          <t>24-sep: borrador completo (10 secciones, Ley 1581 y Decreto 1377, con la autorización de datos sensibles para fotos y selfie) ya en la página. Falta que la cooperativa dé NIT/dirección/ciudad (P-75), fecha de vigencia (P-76), país o región de los servidores (P-77), alternativa sin selfie (P-78), plazos de conservación (P-79) y si reportan a centrales de riesgo Ley 1266 (P-80); y que un abogado la revise (P-81). Bloquea el despliegue (6.5).</t>
         </is>
       </c>
     </row>
@@ -36130,7 +36487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36189,22 +36546,22 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Sebas (acuerdo con Carlos Pardo)</t>
+          <t>sesión principal (coordinador)</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>4.1, 4.7, 4.8, 5.9, 5.10, 6.14, 6.15; P-65 a P-74</t>
+          <t>5.4, P-14, P-61, P-62, P-72; nuevos P-75 a P-81</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Corrección de 4.1 y encargo externo a Carlos Pardo (500.000 COP) por PR a develop</t>
+          <t>Borrador de la política de datos y plantillas de Resend listas; Test QA borrado y dominio conectado</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>4.1 corregida: su texto decía «listado de solicitudes y asociados» pero /admin no tiene lista de asociados ni dashboard, solo afiliaciones, créditos, asesores y sorteo; queda Hecho con el texto correcto. Se contrata a Carlos Pardo, desarrollador externo, para un paquete de 6 actividades que entregará por PR a develop desde su propia rama (cada PR lo revisa un agente ga-* antes de fusionar): 4.7 dashboard de clientes en /admin (peso 4), 4.8 dashboard del asesor en /asesor sin datos sensibles (peso 3), 5.9 convenios administrables desde /admin (peso 3), 5.10 Ley 1581 (borrado automático de fotos rechazadas y motivo de rechazo, peso 2), 6.14 pruebas en celulares reales con informe (peso 1) y 6.15 actualizar los tests e2e viejos al formato de máscara nuevo (peso 1); pendientes P-66 a P-71 en espejo. Nuevos pendientes para Sebas: P-72 (dar acceso de colaborador en GitHub, sin llaves de producción) y P-73 (revisar y pagar los 500.000 COP al fusionar el paquete en develop). P-65 se cierra como Hecho: se decidió que solo participan asociados en el sorteo (S-13, ya implementado).</t>
+          <t>Borrador completo de /politica-de-datos (10 secciones, Ley 1581 y Decreto 1377, con la autorización de datos sensibles para las fotos de cédula y la selfie), con los datos que faltan resaltados en la página con &lt;Pendiente&gt;; 5.4 y P-14 actualizan su bloqueo con la lista concreta que falta de la cooperativa: NIT/dirección/ciudad (P-75), fecha de vigencia (P-76), país o región de los servidores -Supabase, Vercel, Resend- (P-77), alternativa sin selfie (P-78), plazos de conservación -fotos ligadas a P-63- (P-79) y si reportan a centrales de riesgo Ley 1266 (P-80); más la revisión de un abogado (P-81, nuevo pendiente para Sebas). HTML de las 4 plantillas de Resend (ingreso aceptado, crédito aprobado, crédito rechazado, boleta del sorteo) listo en docs/resend/, con el mismo diseño del correo del código; P-61 se actualiza con esa nota, falta que Sebas las cree y publique en Resend junto con las variables de Vercel (RESEND_API_KEY, EMAIL_FROM, RESEND_TEMPLATE_*, SITIO_URL=https://www.greenallianceco.com), ya anotadas en P-44. Sebas: plantilla del código puesta en Supabase, dominio www.greenallianceco.com conectado a producción en Vercel, usuario «Test QA» borrado de producción (P-62 pasa a Hecho), primera variable de Vercel corregida y habló con Carlos para darle acceso de colaborador (P-72 pasa a En curso). El logo de los correos da 404 hasta desplegar develop en main (public/logos no está en producción).</t>
         </is>
       </c>
     </row>
@@ -36214,24 +36571,24 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>ga-escritor-tests</t>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Sebas (acuerdo con Carlos Pardo)</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>6.1, P-58</t>
+          <t>4.1, 4.7, 4.8, 5.9, 5.10, 6.14, 6.15; P-65 a P-74</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>tests/e2e/d-afiliacion.spec.ts reescrito para la afiliación v2; bug real encontrado en esquemaAfiliacion</t>
+          <t>Corrección de 4.1 y encargo externo a Carlos Pardo (500.000 COP) por PR a develop</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Reescritura completa de d-afiliacion.spec.ts (nombres/apellidos, institución + correo institucional, Nequi, asesor, 3 fotos con magic bytes y bucket privado): 48 pruebas × 2 proyectos (escritorio/celular) = 96 contra Supabase local, 92 pasan y 4 fallan (2 por proyecto) por un bug real de la app, no de la prueba. Bug reproducido también como prueba unitaria en tests/unit/validaciones.test.ts (falla a propósito, documentando el defecto): nueva actividad 2.13 y pendiente P-74 para ga-funcionalidad-botones. k-roles.spec.ts (referencia) 4/4 en escritorio, tras corregir a mano el estado de una solicitud de ejemplo que había quedado mal de una corrida previa (no se pudo usar supabase db reset por el permiso de la sandbox). npm run test:unit: 307 pasan, 1 falla (la nueva, documentando el bug); npx tsc --noEmit sin errores. Sigue bloqueado correr npm run test:db (pgTAP) por el mismo permiso de sandbox. Queda fuera de esta tarea, y se delega a Carlos Pardo (ver 6.15, P-71), reescribir b-ingreso.spec.ts, i-despliegue.spec.ts y j-produccion.spec.ts al formato nuevo de máscara de correo.</t>
+          <t>4.1 corregida: su texto decía «listado de solicitudes y asociados» pero /admin no tiene lista de asociados ni dashboard, solo afiliaciones, créditos, asesores y sorteo; queda Hecho con el texto correcto. Se contrata a Carlos Pardo, desarrollador externo, para un paquete de 6 actividades que entregará por PR a develop desde su propia rama (cada PR lo revisa un agente ga-* antes de fusionar): 4.7 dashboard de clientes en /admin (peso 4), 4.8 dashboard del asesor en /asesor sin datos sensibles (peso 3), 5.9 convenios administrables desde /admin (peso 3), 5.10 Ley 1581 (borrado automático de fotos rechazadas y motivo de rechazo, peso 2), 6.14 pruebas en celulares reales con informe (peso 1) y 6.15 actualizar los tests e2e viejos al formato de máscara nuevo (peso 1); pendientes P-66 a P-71 en espejo. Nuevos pendientes para Sebas: P-72 (dar acceso de colaborador en GitHub, sin llaves de producción) y P-73 (revisar y pagar los 500.000 COP al fusionar el paquete en develop). P-65 se cierra como Hecho: se decidió que solo participan asociados en el sorteo (S-13, ya implementado).</t>
         </is>
       </c>
     </row>
@@ -36241,24 +36598,24 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Sebas (coordinación con la cooperativa)</t>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>ga-escritor-tests</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>5.3; P-10, P-11, P-12, P-17, P-18, P-38, P-44</t>
+          <t>6.1, P-58</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Datos reales de contacto entregados; se cancela la importación de Excel; 3 admins reales en producción</t>
+          <t>tests/e2e/d-afiliacion.spec.ts reescrito para la afiliación v2; bug real encontrado en esquemaAfiliacion</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>La cooperativa entregó WhatsApp (311 724 1942), correo de soporte (soporte@greenallianceco.com) y tiempo de respuesta («4 horas o menos»): P-10, P-11, P-12 y P-17 pasan a Hecho; 5.3 actualiza su bloqueo (quedan pendientes texto de vigilancia Supersolidaria, fotos/cifras/testimonios, nombres de los grados y estado de desembolso). Decisión de la cooperativa: no habrá importación de Excel de asociados (la afiliación v2 + aprobación en /admin la reemplaza); P-18 y P-38 pasan a Hecho como «ya no aplica», y 4.4 se cierra igual con nota de cancelación. Ya hay 3 administradores reales en producción (Ricardo, Abogados Prieto y Sebas); la cuenta de prueba «Test QA» (1099887766) sigue siendo admin y hay que borrarla (P-62). Nuevos pendientes de alta prioridad para Sebas: aplicar las 9 migraciones de fase 2 y desplegar (P-59), corregir SUPABASE_SERVICE_ROLE_KEY en Vercel (P-60), crear las plantillas en Resend (P-61), borrar Test QA (P-62), preguntas abiertas a la cooperativa (P-63) y abrir el PR de develop a main (P-64); P-44 actualizado con las variables nuevas (SITIO_URL, RESEND_TEMPLATE_SORTEO_BOLETA).</t>
+          <t>Reescritura completa de d-afiliacion.spec.ts (nombres/apellidos, institución + correo institucional, Nequi, asesor, 3 fotos con magic bytes y bucket privado): 48 pruebas × 2 proyectos (escritorio/celular) = 96 contra Supabase local, 92 pasan y 4 fallan (2 por proyecto) por un bug real de la app, no de la prueba. Bug reproducido también como prueba unitaria en tests/unit/validaciones.test.ts (falla a propósito, documentando el defecto): nueva actividad 2.13 y pendiente P-74 para ga-funcionalidad-botones. k-roles.spec.ts (referencia) 4/4 en escritorio, tras corregir a mano el estado de una solicitud de ejemplo que había quedado mal de una corrida previa (no se pudo usar supabase db reset por el permiso de la sandbox). npm run test:unit: 307 pasan, 1 falla (la nueva, documentando el bug); npx tsc --noEmit sin errores. Sigue bloqueado correr npm run test:db (pgTAP) por el mismo permiso de sandbox. Queda fuera de esta tarea, y se delega a Carlos Pardo (ver 6.15, P-71), reescribir b-ingreso.spec.ts, i-despliegue.spec.ts y j-produccion.spec.ts al formato nuevo de máscara de correo.</t>
         </is>
       </c>
     </row>
@@ -36268,24 +36625,24 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>ga-funcionalidad-botones</t>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Sebas (coordinación con la cooperativa)</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>2.12, 4.1, 4.2, 4.5, 4.6, 6.2; P-36, P-37</t>
+          <t>5.3; P-10, P-11, P-12, P-17, P-18, P-38, P-44</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Afiliación v2, panel /admin y correcciones de la auditoría y la revisión de seguridad (F2-01/F2-04, S-01 a S-14)</t>
+          <t>Datos reales de contacto entregados; se cancela la importación de Excel; 3 admins reales en producción</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Según la coordinación del 24-sep y los commits 235ffbe (afiliación v2 con fotos, panel /admin, vista del asesor y sorteo) y a13c2de (arreglos de auditoría y seguridad), en rama develop, sin tocar producción: formulario de afiliación v2 completo (nombres/apellidos, institución con correo institucional, Nequi, asesor, 3 fotos con subida al bucket privado) y panel /admin (listado de solicitudes y afiliaciones, aprobar/rechazar con motivo, correo «Ingreso aceptado»). Correcciones: (1) F2-01/S-01 boleta oculta, migraciones 000600/000700/000800 aplicadas en local y pasadas a RPC (mi_boleta_sorteo, boletas_confirmadas_sorteo), «Reenviar mi boleta» con tope 3/día; (2) fotos comprimidas a JPEG ≤1600px y bodySizeLimit 3mb; (3) magic bytes para validar el tipo real de la foto; (4) número de boleta fuera de los logs en producción, variables de Resend obligatorias en el build; (5) se quitó `workflow` (0 vulnerabilidades altas); (6) update de solicitudes_credito filtra por estado pendiente; (7) SITIO_URL para el correo «Ingreso aceptado»; (8) participarSorteo exige rol asociado; (9) cabeceras Strict-Transport-Security y Permissions-Policy; (10) vista previa /cuenta?sorteo=demo solo fuera de producción; (11) S-06 respuesta idéntica para cédula duplicada en afiliación, sin filtrar si ya existe. Verificación: tsc, eslint, build y test:unit (307/307) sin errores; playwright k-roles (4/4). 4.1, 4.2, 4.5 pasan a Hecho (panel /admin probado). Pendiente: tests/e2e/d-afiliacion.spec.ts desactualizado (ver P-58); variables nuevas de Vercel (ver P-59 a P-61).</t>
+          <t>La cooperativa entregó WhatsApp (311 724 1942), correo de soporte (soporte@greenallianceco.com) y tiempo de respuesta («4 horas o menos»): P-10, P-11, P-12 y P-17 pasan a Hecho; 5.3 actualiza su bloqueo (quedan pendientes texto de vigilancia Supersolidaria, fotos/cifras/testimonios, nombres de los grados y estado de desembolso). Decisión de la cooperativa: no habrá importación de Excel de asociados (la afiliación v2 + aprobación en /admin la reemplaza); P-18 y P-38 pasan a Hecho como «ya no aplica», y 4.4 se cierra igual con nota de cancelación. Ya hay 3 administradores reales en producción (Ricardo, Abogados Prieto y Sebas); la cuenta de prueba «Test QA» (1099887766) sigue siendo admin y hay que borrarla (P-62). Nuevos pendientes de alta prioridad para Sebas: aplicar las 9 migraciones de fase 2 y desplegar (P-59), corregir SUPABASE_SERVICE_ROLE_KEY en Vercel (P-60), crear las plantillas en Resend (P-61), borrar Test QA (P-62), preguntas abiertas a la cooperativa (P-63) y abrir el PR de develop a main (P-64); P-44 actualizado con las variables nuevas (SITIO_URL, RESEND_TEMPLATE_SORTEO_BOLETA).</t>
         </is>
       </c>
     </row>
@@ -36297,22 +36654,22 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ga-revisor-seguridad</t>
+          <t>ga-funcionalidad-botones</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>2.12, 4.1, 4.2, 4.5, 4.6, 6.2; P-36, P-37</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Revisión de seguridad de fase 2: 3 bloqueos para el despliegue</t>
+          <t>Afiliación v2, panel /admin y correcciones de la auditoría y la revisión de seguridad (F2-01/F2-04, S-01 a S-14)</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Diff 4545c0e..235ffbe (/admin, /asesor, /afiliacion v2, sorteo, proxy, ingreso por rol, cabeceras, llaves). Sin secretos expuestos, open redirect ni bypass de rol; /admin y /asesor verifican el rol en el servidor antes de usar service role. Bloquean el despliegue: (1) F2-01 boleta legible por API REST (ya reportado por ga-auditor-supabase); (2) la autorización de datos sensibles enlaza a una política de datos todavía placeholder; (3) el límite de 1 MB de las Server Actions tumba el envío de las 3 fotos. 6.2 sigue En curso (pasa a depender también de 2.12, 3.9 y 4.6): la mayoría de estos hallazgos ya se corrigieron en el siguiente reporte, falta el visto bueno final. Nuevo pendiente P-65 (si admin o asesor pueden participar en el sorteo).</t>
+          <t>Según la coordinación del 24-sep y los commits 235ffbe (afiliación v2 con fotos, panel /admin, vista del asesor y sorteo) y a13c2de (arreglos de auditoría y seguridad), en rama develop, sin tocar producción: formulario de afiliación v2 completo (nombres/apellidos, institución con correo institucional, Nequi, asesor, 3 fotos con subida al bucket privado) y panel /admin (listado de solicitudes y afiliaciones, aprobar/rechazar con motivo, correo «Ingreso aceptado»). Correcciones: (1) F2-01/S-01 boleta oculta, migraciones 000600/000700/000800 aplicadas en local y pasadas a RPC (mi_boleta_sorteo, boletas_confirmadas_sorteo), «Reenviar mi boleta» con tope 3/día; (2) fotos comprimidas a JPEG ≤1600px y bodySizeLimit 3mb; (3) magic bytes para validar el tipo real de la foto; (4) número de boleta fuera de los logs en producción, variables de Resend obligatorias en el build; (5) se quitó `workflow` (0 vulnerabilidades altas); (6) update de solicitudes_credito filtra por estado pendiente; (7) SITIO_URL para el correo «Ingreso aceptado»; (8) participarSorteo exige rol asociado; (9) cabeceras Strict-Transport-Security y Permissions-Policy; (10) vista previa /cuenta?sorteo=demo solo fuera de producción; (11) S-06 respuesta idéntica para cédula duplicada en afiliación, sin filtrar si ya existe. Verificación: tsc, eslint, build y test:unit (307/307) sin errores; playwright k-roles (4/4). 4.1, 4.2, 4.5 pasan a Hecho (panel /admin probado). Pendiente: tests/e2e/d-afiliacion.spec.ts desactualizado (ver P-58); variables nuevas de Vercel (ver P-59 a P-61).</t>
         </is>
       </c>
     </row>
@@ -36324,22 +36681,22 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ga-auditor-supabase</t>
+          <t>ga-revisor-seguridad</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Auditoría de las 6 migraciones de fase 2: 1 hallazgo alto, 3 migraciones correctivas propuestas</t>
+          <t>Revisión de seguridad de fase 2: 3 bloqueos para el despliegue</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Auditoría de solo lectura contra el repo y Supabase local (203/203 pgTAP). Sin nada crítico. Hallazgo alto: el asociado podía leer el número de su boleta del sorteo por la API REST antes de confirmarlo. 3 migraciones nuevas propuestas sin aplicar: 000600 (oculta el número y corrige las carreras del sorteo), 000700 (el asesor degradado deja de ver a sus clientes), 000800 (trigger que sincroniza cédula y grado desde app_metadata). Reporte: docs/auditorias/2026-09-24-fase-2.md. Nueva actividad 1.6 (peso 3, depende de 1.5).</t>
+          <t>Diff 4545c0e..235ffbe (/admin, /asesor, /afiliacion v2, sorteo, proxy, ingreso por rol, cabeceras, llaves). Sin secretos expuestos, open redirect ni bypass de rol; /admin y /asesor verifican el rol en el servidor antes de usar service role. Bloquean el despliegue: (1) F2-01 boleta legible por API REST (ya reportado por ga-auditor-supabase); (2) la autorización de datos sensibles enlaza a una política de datos todavía placeholder; (3) el límite de 1 MB de las Server Actions tumba el envío de las 3 fotos. 6.2 sigue En curso (pasa a depender también de 2.12, 3.9 y 4.6): la mayoría de estos hallazgos ya se corrigieron en el siguiente reporte, falta el visto bueno final. Nuevo pendiente P-65 (si admin o asesor pueden participar en el sorteo).</t>
         </is>
       </c>
     </row>
@@ -36351,22 +36708,22 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ga-funcionalidad-botones</t>
+          <t>ga-auditor-supabase</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Sorteo mensual en /cuenta</t>
+          <t>Auditoría de las 6 migraciones de fase 2: 1 hallazgo alto, 3 migraciones correctivas propuestas</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Botón «Sorteo del mes» y modal en /cuenta (components/sorteo/SorteoDelMes.tsx): participar (RPC participar_sorteo, correo con el número por Resend), confirmar (RPC confirmar_boleta_sorteo, tope 5 intentos) y celebración con confeti (respeta prefers-reduced-motion). El número de boleta nunca sale del servidor antes de confirmar. 31 pruebas unitarias nuevas; docs/mapa-de-botones.md §4 y .env.example (RESEND_TEMPLATE_SORTEO_BOLETA) actualizados. tsc, eslint y build sin errores nuevos. No se pudo probar el flujo feliz completo en vivo (24-sep está fuera de la ventana 1–5); cubierto con pruebas unitarias y revisión de código. Nueva actividad 3.9 (peso 4, depende de 3.5 y 1.5). Pendiente: aprobar la plantilla ga-sorteo-boleta en Resend (ver P-61).</t>
+          <t>Auditoría de solo lectura contra el repo y Supabase local (203/203 pgTAP). Sin nada crítico. Hallazgo alto: el asociado podía leer el número de su boleta del sorteo por la API REST antes de confirmarlo. 3 migraciones nuevas propuestas sin aplicar: 000600 (oculta el número y corrige las carreras del sorteo), 000700 (el asesor degradado deja de ver a sus clientes), 000800 (trigger que sincroniza cédula y grado desde app_metadata). Reporte: docs/auditorias/2026-09-24-fase-2.md. Nueva actividad 1.6 (peso 3, depende de 1.5).</t>
         </is>
       </c>
     </row>
@@ -36383,17 +36740,17 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>4.6; P-57</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Rol asesor: /asesor (mis clientes) y /asesor/demo</t>
+          <t>Sorteo mensual en /cuenta</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>/asesor («Mis clientes», buscador y filtro por estado sobre resumen_clientes_asesor()) y /asesor/demo (cuenta fantasma que no escribe nada), ambas con guardia de rol propia en el servidor; 26 pruebas unitarias nuevas; docs/mapa-de-botones.md actualizado (§7, §7b). Verificado contra Supabase local con el asesor de prueba (cédula 1234567892). Nueva actividad 4.6 (peso 3, depende de 1.5). Pendiente nuevo P-57: agregar /asesor al matcher de proxy.ts y redirigir por rol tras login.</t>
+          <t>Botón «Sorteo del mes» y modal en /cuenta (components/sorteo/SorteoDelMes.tsx): participar (RPC participar_sorteo, correo con el número por Resend), confirmar (RPC confirmar_boleta_sorteo, tope 5 intentos) y celebración con confeti (respeta prefers-reduced-motion). El número de boleta nunca sale del servidor antes de confirmar. 31 pruebas unitarias nuevas; docs/mapa-de-botones.md §4 y .env.example (RESEND_TEMPLATE_SORTEO_BOLETA) actualizados. tsc, eslint y build sin errores nuevos. No se pudo probar el flujo feliz completo en vivo (24-sep está fuera de la ventana 1–5); cubierto con pruebas unitarias y revisión de código. Nueva actividad 3.9 (peso 4, depende de 3.5 y 1.5). Pendiente: aprobar la plantilla ga-sorteo-boleta en Resend (ver P-61).</t>
         </is>
       </c>
     </row>
@@ -36405,49 +36762,49 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ga-auditor-supabase</t>
+          <t>ga-funcionalidad-botones</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>1.5; P-63</t>
+          <t>4.6; P-57</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Modelo de datos de fase 2: rol asesor, afiliación v2, bucket de fotos y sorteo mensual</t>
+          <t>Rol asesor: /asesor (mis clientes) y /asesor/demo</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>6 migraciones nuevas probadas contra Supabase local (no aplicadas a producción): enum 'asesor', perfiles.asesor_id con validaciones, solicitudes_afiliacion v2 (nombres/apellidos, institución + correo institucional, Nequi, asesor_id, 3 fotos obligatorias), obtener_asesores_publico()/resumen_clientes_asesor() (SECURITY DEFINER), bucket privado afiliacion-documentos (5 MB, sin políticas de storage.objects, todo por service_role + URL firmada) y sorteo mensual (boletas_sorteo, participar_sorteo(), confirmar_boleta_sorteo(), ventana 1–5 hora Bogotá, tope 5 intentos). seed.sql actualizado; 4 archivos pgTAP nuevos y 2 ajustados; docs/spec-fase-2.md nuevo. Verificado: supabase db reset + supabase test db (203/203) + test:unit (163/163) + tsc sin errores. Nueva actividad 1.5 (peso 5, depende de 1.2). Pendientes abiertos para la cooperativa recogidos en P-63.</t>
+          <t>/asesor («Mis clientes», buscador y filtro por estado sobre resumen_clientes_asesor()) y /asesor/demo (cuenta fantasma que no escribe nada), ambas con guardia de rol propia en el servidor; 26 pruebas unitarias nuevas; docs/mapa-de-botones.md actualizado (§7, §7b). Verificado contra Supabase local con el asesor de prueba (cédula 1234567892). Nueva actividad 4.6 (peso 3, depende de 1.5). Pendiente nuevo P-57: agregar /asesor al matcher de proxy.ts y redirigir por rol tras login.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>ga-funcionalidad-botones + ga-diseno-a-codigo</t>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>ga-auditor-supabase</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>1.5; P-63</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Corregidos F-01 a F-08 de verificación 3 y los 8 hallazgos responsive</t>
+          <t>Modelo de datos de fase 2: rol asesor, afiliación v2, bucket de fotos y sorteo mensual</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>ga-funcionalidad-botones: F-01 (correo enmascarado ya no delata la cédula, también oculta el dominio), F-02 (tope de intentos al verificar código: 5 por cédula y 30 por IP cada 15 min), F-05 (cabeceras X-Frame-Options, CSP frame-ancestors, Referrer-Policy, X-Content-Type-Options), F-06 (monto múltiplo de $50.000) y F-08 (código pegado durante «Reenviar» ya no se borra); documentó O-01 (x-forwarded-for solo confiable detrás de Vercel, ver P-49). ga-diseno-a-codigo: los 8 hallazgos responsive (tarjetas 50/100 %, deslizador, «Reenviar código», header /cuenta, hero y landing 1024–1150, /afiliacion y /cuenta 640–1023, hueco /afiliacion/enviada en tableta) y F-03/F-04/F-07 (Cerrar sesión en celular, 404 en español, hueco de tableta); nueva app/not-found.tsx. Todo terminó en el commit bf09975→4545c0e (arreglos de QA). Pendiente: tests/e2e con el formato viejo de máscara y dominios (ver P-58); confirmar con la cooperativa que solo hay 3 dominios institucionales (ver P-63); hallazgo #7 (grid de /afiliacion a 1024 px) quedó pendiente para la tanda que reescribiera Afiliacion.tsx, ya superado por la afiliación v2 (2.12).</t>
+          <t>6 migraciones nuevas probadas contra Supabase local (no aplicadas a producción): enum 'asesor', perfiles.asesor_id con validaciones, solicitudes_afiliacion v2 (nombres/apellidos, institución + correo institucional, Nequi, asesor_id, 3 fotos obligatorias), obtener_asesores_publico()/resumen_clientes_asesor() (SECURITY DEFINER), bucket privado afiliacion-documentos (5 MB, sin políticas de storage.objects, todo por service_role + URL firmada) y sorteo mensual (boletas_sorteo, participar_sorteo(), confirmar_boleta_sorteo(), ventana 1–5 hora Bogotá, tope 5 intentos). seed.sql actualizado; 4 archivos pgTAP nuevos y 2 ajustados; docs/spec-fase-2.md nuevo. Verificado: supabase db reset + supabase test db (203/203) + test:unit (163/163) + tsc sin errores. Nueva actividad 1.5 (peso 5, depende de 1.2). Pendientes abiertos para la cooperativa recogidos en P-63.</t>
         </is>
       </c>
     </row>
@@ -36459,22 +36816,22 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>ga-verificador-responsive + ga-verificador-qa</t>
+          <t>ga-funcionalidad-botones + ga-diseno-a-codigo</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>6.3; P-39</t>
+          <t>6.3</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Responsive 3 (8 hallazgos menores) y QA E2E 3 (236/241, NO APROBADO)</t>
+          <t>Corregidos F-01 a F-08 de verificación 3 y los 8 hallazgos responsive</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Responsive: 8 rutas × 9 anchos (360–1440) contra develop bf09975, 0 críticos y 8 menores (docs/verificaciones/responsive-2026-09-23/). QA: Supabase local, 236 pasan y 5 fallan; unitarias (140), pgTAP (143), tsc y eslint sin errores; docs/verificaciones/2026-09-23-verificacion-3.md. Bloqueaban producción: F-01 crítica (el dominio del correo enmascarado delataba si la cédula existe) y F-02 alta (sin tope de intentos al verificar el código); además contenido pendiente de la cooperativa, política de datos vacía, configuración de producción por revisar (SMTP/Resend, P-45, secretos en Vercel, P-43, P-09), F-03/F-04 (diseño), F-05 (cabeceras anti-clickjacking) y F-06 a F-08 bajas.</t>
+          <t>ga-funcionalidad-botones: F-01 (correo enmascarado ya no delata la cédula, también oculta el dominio), F-02 (tope de intentos al verificar código: 5 por cédula y 30 por IP cada 15 min), F-05 (cabeceras X-Frame-Options, CSP frame-ancestors, Referrer-Policy, X-Content-Type-Options), F-06 (monto múltiplo de $50.000) y F-08 (código pegado durante «Reenviar» ya no se borra); documentó O-01 (x-forwarded-for solo confiable detrás de Vercel, ver P-49). ga-diseno-a-codigo: los 8 hallazgos responsive (tarjetas 50/100 %, deslizador, «Reenviar código», header /cuenta, hero y landing 1024–1150, /afiliacion y /cuenta 640–1023, hueco /afiliacion/enviada en tableta) y F-03/F-04/F-07 (Cerrar sesión en celular, 404 en español, hueco de tableta); nueva app/not-found.tsx. Todo terminó en el commit bf09975→4545c0e (arreglos de QA). Pendiente: tests/e2e con el formato viejo de máscara y dominios (ver P-58); confirmar con la cooperativa que solo hay 3 dominios institucionales (ver P-63); hallazgo #7 (grid de /afiliacion a 1024 px) quedó pendiente para la tanda que reescribiera Afiliacion.tsx, ya superado por la afiliación v2 (2.12).</t>
         </is>
       </c>
     </row>
@@ -36484,24 +36841,24 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>ga-verificador-responsive</t>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>ga-verificador-responsive + ga-verificador-qa</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>6.3, 5.2, 5.8; P-39, P-53</t>
+          <t>6.3; P-39</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Verificación responsive 2: 0 fallas en 13 anchos; tests/responsive 10/10</t>
+          <t>Responsive 3 (8 hallazgos menores) y QA E2E 3 (236/241, NO APROBADO)</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Sin scroll horizontal en /, /ingresar, /ingresar/codigo, /afiliacion, /politica-de-datos, /cuenta y /cuenta/solicitar (con cookie y sesión reales) de 320 a 1920 px. P-39 pasa a Hecho (QA y responsive corridas); 6.3 sigue En curso porque depende de trabajo sin terminar. Menor y opcional: P-53 («COOPERATIVA» del logo a 320 px ~5 px de alto).</t>
+          <t>Responsive: 8 rutas × 9 anchos (360–1440) contra develop bf09975, 0 críticos y 8 menores (docs/verificaciones/responsive-2026-09-23/). QA: Supabase local, 236 pasan y 5 fallan; unitarias (140), pgTAP (143), tsc y eslint sin errores; docs/verificaciones/2026-09-23-verificacion-3.md. Bloqueaban producción: F-01 crítica (el dominio del correo enmascarado delataba si la cédula existe) y F-02 alta (sin tope de intentos al verificar el código); además contenido pendiente de la cooperativa, política de datos vacía, configuración de producción por revisar (SMTP/Resend, P-45, secretos en Vercel, P-43, P-09), F-03/F-04 (diseño), F-05 (cabeceras anti-clickjacking) y F-06 a F-08 bajas.</t>
         </is>
       </c>
     </row>
@@ -36513,22 +36870,22 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>ga-funcionalidad-botones</t>
+          <t>ga-verificador-responsive</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>3.7, 5.5, 5.6, 6.9, 6.11; P-35, P-40, P-44, P-56</t>
+          <t>6.3, 5.2, 5.8; P-39, P-53</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>HMAC en el límite de intentos, crédito en /cuenta/solicitar y borradas /login y /dashboard</t>
+          <t>Verificación responsive 2: 0 fallas en 13 anchos; tests/responsive 10/10</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Nueva actividad 6.11 (Hecho, peso 1): clave del límite con HMAC-SHA256 y LIMITE_HMAC_SECRET (sin el secreto el build falla). Formulario de crédito movido a /cuenta/solicitar con EncabezadoCuenta; 5.5 y P-40 pasan a Hecho. 6.9 y P-44 suman LIMITE_HMAC_SECRET y 6.9 depende de 6.11. Pruebas: 140/140 unitarias, 143/143 base, tsc, lint y build limpios. Trabajo nuevo: 5.6 revisar el diseño de /cuenta/solicitar (ga-diseno-a-codigo, peso 1) con P-56; 6.3 pasa a depender de 5.6.</t>
+          <t>Sin scroll horizontal en /, /ingresar, /ingresar/codigo, /afiliacion, /politica-de-datos, /cuenta y /cuenta/solicitar (con cookie y sesión reales) de 320 a 1920 px. P-39 pasa a Hecho (QA y responsive corridas); 6.3 sigue En curso porque depende de trabajo sin terminar. Menor y opcional: P-53 («COOPERATIVA» del logo a 320 px ~5 px de alto).</t>
         </is>
       </c>
     </row>
@@ -36540,22 +36897,22 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>ga-diseno-a-codigo</t>
+          <t>ga-funcionalidad-botones</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>5.2, 5.8, 6.3</t>
+          <t>3.7, 5.5, 5.6, 6.9, 6.11; P-35, P-40, P-44, P-56</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Corregido el scroll horizontal y marca de agua más tenue</t>
+          <t>HMAC en el límite de intentos, crédito en /cuenta/solicitar y borradas /login y /dashboard</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Enlace del logo encoge (min-w-0 shrink) en los 5 headers; formulario de ingreso w-full con máximo 440 px y relleno de 32 px entre 1024 y 1279 px; marca de agua del hero en la esquina contraria y más tenue. 5.8 queda Hecho (peso 1, depende de 5.2 y 5.7).</t>
+          <t>Nueva actividad 6.11 (Hecho, peso 1): clave del límite con HMAC-SHA256 y LIMITE_HMAC_SECRET (sin el secreto el build falla). Formulario de crédito movido a /cuenta/solicitar con EncabezadoCuenta; 5.5 y P-40 pasan a Hecho. 6.9 y P-44 suman LIMITE_HMAC_SECRET y 6.9 depende de 6.11. Pruebas: 140/140 unitarias, 143/143 base, tsc, lint y build limpios. Trabajo nuevo: 5.6 revisar el diseño de /cuenta/solicitar (ga-diseno-a-codigo, peso 1) con P-56; 6.3 pasa a depender de 5.6.</t>
         </is>
       </c>
     </row>
@@ -36567,22 +36924,22 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>ga-verificador-responsive</t>
+          <t>ga-diseno-a-codigo</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>6.3, 5.2, 2.1, 5.8; P-39</t>
+          <t>5.2, 5.8, 6.3</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Verificación responsive 1: logo y fotos bien; 2 fallas críticas de scroll previas</t>
+          <t>Corregido el scroll horizontal y marca de agua más tenue</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Playwright en 10 anchos (320–1920 px) sobre 7 rutas. Logo nítido y proporcionado en dark y light; fotos decorativas correctas. Fallas: landing a 320 px («Ingresar» cortado, enlace del logo fijo en 240 px) y /ingresar y /ingresar/codigo entre 1024 y 1075 px (540 + 440 + padding = 1076 px). Se abre 5.8 para corregirlas.</t>
+          <t>Enlace del logo encoge (min-w-0 shrink) en los 5 headers; formulario de ingreso w-full con máximo 440 px y relleno de 32 px entre 1024 y 1279 px; marca de agua del hero en la esquina contraria y más tenue. 5.8 queda Hecho (peso 1, depende de 5.2 y 5.7).</t>
         </is>
       </c>
     </row>
@@ -36594,22 +36951,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>ga-diseno-a-codigo</t>
+          <t>ga-verificador-responsive</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>2.1, 5.3, 5.7; P-16, P-52</t>
+          <t>6.3, 5.2, 2.1, 5.8; P-39</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Logo con letras oficiales en SVG y espacios de foto de marca en la landing</t>
+          <t>Verificación responsive 1: logo y fotos bien; 2 fallas críticas de scroll previas</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>green-alliance-wordmark.svg (y versión blanca) reemplaza Montserrat; EspacioFoto con degradado, patrón, isotipo e ilustración, listo para recibir { src, alt }. Mapa de botones revisado contra el diseño (2.2, 2.3, 3.4): todo existe y está bien ubicado. Nueva actividad 5.7 (Hecho, peso 2, depende de 2.1). 5.3 sigue Bloqueado; P-16 sigue Pendiente (fotos reales de la cooperativa). P-52 (actualizar el mapa: §4 «Nueva solicitud» → /cuenta/solicitar y documentar esa ruta) se registra como Hecho: el documento ya lo tiene tras el cambio de ga-funcionalidad-botones.</t>
+          <t>Playwright en 10 anchos (320–1920 px) sobre 7 rutas. Logo nítido y proporcionado en dark y light; fotos decorativas correctas. Fallas: landing a 320 px («Ingresar» cortado, enlace del logo fijo en 240 px) y /ingresar y /ingresar/codigo entre 1024 y 1075 px (540 + 440 + padding = 1076 px). Se abre 5.8 para corregirlas.</t>
         </is>
       </c>
     </row>
@@ -36621,22 +36978,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>ga-auditor-supabase</t>
+          <t>ga-diseno-a-codigo</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>6.8, 6.11, 6.12; P-43, P-54, P-55</t>
+          <t>2.1, 5.3, 5.7; P-16, P-52</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Migración limite_de_intentos auditada: se puede aplicar tal cual</t>
+          <t>Logo con letras oficiales en SVG y espacios de foto de marca en la landing</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Auditoría de solo lectura contra producción, sin críticos ni altos (docs/auditorias/2026-09-23-limite-de-intentos.md). 6.8 pasa a En curso (revisión hecha, falta que Sebas haga db push antes de 6.5); P-43 sigue Pendiente con nota. Trabajo nuevo: hash HMAC de la clave (queda en 6.11, ver reporte de ga-funcionalidad-botones), 6.12 alerta en logs de Vercel (peso 1) con P-54, y P-55 opcional (revocar limites_intentos_id_seq a anon y authenticated).</t>
+          <t>green-alliance-wordmark.svg (y versión blanca) reemplaza Montserrat; EspacioFoto con degradado, patrón, isotipo e ilustración, listo para recibir { src, alt }. Mapa de botones revisado contra el diseño (2.2, 2.3, 3.4): todo existe y está bien ubicado. Nueva actividad 5.7 (Hecho, peso 2, depende de 2.1). 5.3 sigue Bloqueado; P-16 sigue Pendiente (fotos reales de la cooperativa). P-52 (actualizar el mapa: §4 «Nueva solicitud» → /cuenta/solicitar y documentar esa ruta) se registra como Hecho: el documento ya lo tiene tras el cambio de ga-funcionalidad-botones.</t>
         </is>
       </c>
     </row>
@@ -36646,24 +37003,24 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Sebas + ga-auditor-supabase</t>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>ga-auditor-supabase</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>2.4, 6.8, 6.10; P-09, P-19, P-20, P-43, P-45</t>
+          <t>6.8, 6.11, 6.12; P-43, P-54, P-55</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>SMTP de Resend configurado, plantilla del código lista en local y blindar confirmada en producción</t>
+          <t>Migración limite_de_intentos auditada: se puede aplicar tal cual</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>P-19 Hecho (Sebas configuró el SMTP). P-20 sigue En curso: supabase/templates/codigo-ingreso.html rediseñada con la marca y probada en Mailpit; falta pegarla en Magic Link del panel. P-45 sin confirmar, sin cambios; por eso 2.4 sigue En curso. list_migrations confirma que producción ya tiene 20260923173355_blindar_solicitudes_y_revisiones: 6.10 y P-09 pasan a Hecho (el reporte anterior de atraso estaba equivocado). Falta en producción 20260923210000_limite_de_intentos (limites_intentos y registrar_intento, usadas por dentroDelLimite en /afiliacion, /ingresar y «Reenviar código»): ya existía como 6.8 / P-43 y 6.5 ya dependía de 6.8; se actualizan responsable (Sebas, revisa ga-auditor-supabase) y nota en vez de duplicar.</t>
+          <t>Auditoría de solo lectura contra producción, sin críticos ni altos (docs/auditorias/2026-09-23-limite-de-intentos.md). 6.8 pasa a En curso (revisión hecha, falta que Sebas haga db push antes de 6.5); P-43 sigue Pendiente con nota. Trabajo nuevo: hash HMAC de la clave (queda en 6.11, ver reporte de ga-funcionalidad-botones), 6.12 alerta en logs de Vercel (peso 1) con P-54, y P-55 opcional (revocar limites_intentos_id_seq a anon y authenticated).</t>
         </is>
       </c>
     </row>
@@ -36673,24 +37030,24 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Sebas</t>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Sebas + ga-auditor-supabase</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2.4, 6.8, 6.10; P-09, P-19, P-20, P-43, P-45</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Agente ga-auditor-supabase corregido</t>
+          <t>SMTP de Resend configurado, plantilla del código lista en local y blindar confirmada en producción</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Sus disallowedTools ahora usan los nombres reales del MCP (mcp__claude_ai_Supabase__*). Sin efecto en el plan.</t>
+          <t>P-19 Hecho (Sebas configuró el SMTP). P-20 sigue En curso: supabase/templates/codigo-ingreso.html rediseñada con la marca y probada en Mailpit; falta pegarla en Magic Link del panel. P-45 sin confirmar, sin cambios; por eso 2.4 sigue En curso. list_migrations confirma que producción ya tiene 20260923173355_blindar_solicitudes_y_revisiones: 6.10 y P-09 pasan a Hecho (el reporte anterior de atraso estaba equivocado). Falta en producción 20260923210000_limite_de_intentos (limites_intentos y registrar_intento, usadas por dentroDelLimite en /afiliacion, /ingresar y «Reenviar código»): ya existía como 6.8 / P-43 y 6.5 ya dependía de 6.8; se actualizan responsable (Sebas, revisa ga-auditor-supabase) y nota en vez de duplicar.</t>
         </is>
       </c>
     </row>
@@ -36700,24 +37057,24 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Sebas + ga-auditor-supabase</t>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Sebas</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>3.1, 6.5, 6.10; P-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Producción atrasada: falta la migración blindar_solicitudes_y_revisiones</t>
+          <t>Agente ga-auditor-supabase corregido</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>PagGreenAlliance tiene 10 migraciones hasta 20260923123937_fecha_solicitud_en_servidor; le falta blindar_solicitudes_y_revisiones (en el repo es 20260923173355; el reporte la nombra 20260923160000) y la app lee tasa_interes_mensual, que en producción no existe. P-09 estaba Hecho por error: se reabre como Pendiente Alta (Sebas aplica, ga-auditor-supabase revisa antes). 3.1 se deja Hecho (el trabajo en la base está hecho y tiene hechas que dependen de él) pero se quita «y migración a producción» de su texto; nueva actividad 6.10 (peso 1, depende de 3.1) para aplicarla, y 6.5 (despliegue) pasa a depender de 6.10.</t>
+          <t>Sus disallowedTools ahora usan los nombres reales del MCP (mcp__claude_ai_Supabase__*). Sin efecto en el plan.</t>
         </is>
       </c>
     </row>
@@ -36727,24 +37084,24 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>ga-escritor-tests</t>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Sebas + ga-auditor-supabase</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.1, 6.5, 6.10; P-09</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>132/132 unitarias, 131/131 pgTAP y tsc sin errores</t>
+          <t>Producción atrasada: falta la migración blindar_solicitudes_y_revisiones</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Corridas con Node v24 y Supabase local en Docker. Se agregaron supabase/seed.sql con asociados de prueba y .env.development.local para que npm run dev use Supabase local en vez de producción. 6.1 sigue En curso: faltan las pruebas de las acciones de admin (4.3, 4.5).</t>
+          <t>PagGreenAlliance tiene 10 migraciones hasta 20260923123937_fecha_solicitud_en_servidor; le falta blindar_solicitudes_y_revisiones (en el repo es 20260923173355; el reporte la nombra 20260923160000) y la app lee tasa_interes_mensual, que en producción no existe. P-09 estaba Hecho por error: se reabre como Pendiente Alta (Sebas aplica, ga-auditor-supabase revisa antes). 3.1 se deja Hecho (el trabajo en la base está hecho y tiene hechas que dependen de él) pero se quita «y migración a producción» de su texto; nueva actividad 6.10 (peso 1, depende de 3.1) para aplicarla, y 6.5 (despliegue) pasa a depender de 6.10.</t>
         </is>
       </c>
     </row>
@@ -36754,24 +37111,24 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Sebas + ga-funcionalidad-botones</t>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>ga-escritor-tests</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>2.9, 3.8, 4.5, 6.1, 6.2, 6.9; P-19, P-20, P-28, P-36, P-37, P-44, P-45, P-50, P-51</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Se quitan del código los correos de aviso de afiliación y de solicitud de crédito; docs/resend-plantillas.md reescrito</t>
+          <t>132/132 unitarias, 131/131 pgTAP y tsc sin errores</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>Decisión de Sebas: ya no se envían avisos Resend al guardar una afiliación (equipo y solicitante) ni una solicitud de crédito (equipo y asociado). Se borró lib/correo/afiliacion.ts y enviarAvisoNuevaSolicitudCredito; salen del .env.example AFILIACION_EMAIL_EQUIPO, CREDITOS_EMAIL_EQUIPO y cuatro RESEND_TEMPLATE_*, entra RESEND_TEMPLATE_INGRESO_ACEPTADO. El equipo revisa solicitudes y afiliaciones en Supabase hasta que exista /admin. Se elimina la actividad 3.8 (correo al equipo, estaba En curso, peso 2) y se quita de las dependencias de 6.1 y 6.2. 2.9 y P-28 ya no mencionan el correo. 6.9 y P-44: fuera AFILIACION_EMAIL_EQUIPO, entran RESEND_TEMPLATE_INGRESO_ACEPTADO, _CREDITO_APROBADO y _CREDITO_RECHAZADO. Plantillas: (a) «Ingreso aceptado» → nueva actividad 4.5 (aprobar afiliación en /admin, crear usuario y enviar correo; peso 3, depende de 4.1 y 2.9; 6.1 y 6.2 pasan a depender de ella) y pendiente P-51; (b) código de 6 dígitos lo envía Supabase Auth, funciona en local, en producción falta SMTP de Resend, plantilla Magic Link con {{ .Token }}, OTP de 6 dígitos y 600 s → se actualizan P-19, P-20 y P-45 (responsable «Yo (panel Supabase/Resend)»), ligados a 2.4; (c) «Resultado del crédito»: enviarResultadoCredito existe sin conectar → P-37 se redefine y pasa a 4.3. P-50 queda Hecho como «ya no aplica».</t>
+          <t>Corridas con Node v24 y Supabase local en Docker. Se agregaron supabase/seed.sql con asociados de prueba y .env.development.local para que npm run dev use Supabase local en vez de producción. 6.1 sigue En curso: faltan las pruebas de las acciones de admin (4.3, 4.5).</t>
         </is>
       </c>
     </row>
@@ -36781,24 +37138,24 @@
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>ga-verificador-qa</t>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Sebas + ga-funcionalidad-botones</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>6.3, 2.11; P-39, P-48, P-49, P-50</t>
+          <t>2.9, 3.8, 4.5, 6.1, 6.2, 6.9; P-19, P-20, P-28, P-36, P-37, P-44, P-45, P-50, P-51</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>QA 1 de punta a punta: 186 pruebas pasan, 2 fallan</t>
+          <t>Se quitan del código los correos de aviso de afiliación y de solicitud de crédito; docs/resend-plantillas.md reescrito</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Playwright contra Supabase local (1280 y 390 px); pruebas en tests/e2e/ e informe en docs/verificaciones/2026-09-23-verificacion-1.md. Sin fallas críticas ni altas; una media (F-01: el select «Grado» de /afiliacion se vacía tras un error de validación). 6.3 y P-39 pasan a En curso (falta ga-verificador-responsive). Nueva actividad 2.11 (corregir F-01, peso 1, depende de 2.9) y 6.3 pasa a depender de ella. Pendientes nuevos: P-48 (F-01), P-49 (revisar x-forwarded-for para el límite por IP, ligado a 6.2) y P-50 (confirmar el envío de los correos de afiliación, ligado a 3.8).</t>
+          <t>Decisión de Sebas: ya no se envían avisos Resend al guardar una afiliación (equipo y solicitante) ni una solicitud de crédito (equipo y asociado). Se borró lib/correo/afiliacion.ts y enviarAvisoNuevaSolicitudCredito; salen del .env.example AFILIACION_EMAIL_EQUIPO, CREDITOS_EMAIL_EQUIPO y cuatro RESEND_TEMPLATE_*, entra RESEND_TEMPLATE_INGRESO_ACEPTADO. El equipo revisa solicitudes y afiliaciones en Supabase hasta que exista /admin. Se elimina la actividad 3.8 (correo al equipo, estaba En curso, peso 2) y se quita de las dependencias de 6.1 y 6.2. 2.9 y P-28 ya no mencionan el correo. 6.9 y P-44: fuera AFILIACION_EMAIL_EQUIPO, entran RESEND_TEMPLATE_INGRESO_ACEPTADO, _CREDITO_APROBADO y _CREDITO_RECHAZADO. Plantillas: (a) «Ingreso aceptado» → nueva actividad 4.5 (aprobar afiliación en /admin, crear usuario y enviar correo; peso 3, depende de 4.1 y 2.9; 6.1 y 6.2 pasan a depender de ella) y pendiente P-51; (b) código de 6 dígitos lo envía Supabase Auth, funciona en local, en producción falta SMTP de Resend, plantilla Magic Link con {{ .Token }}, OTP de 6 dígitos y 600 s → se actualizan P-19, P-20 y P-45 (responsable «Yo (panel Supabase/Resend)»), ligados a 2.4; (c) «Resultado del crédito»: enviarResultadoCredito existe sin conectar → P-37 se redefine y pasa a 4.3. P-50 queda Hecho como «ya no aplica».</t>
         </is>
       </c>
     </row>
@@ -36810,22 +37167,22 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>ga-funcionalidad-botones</t>
+          <t>ga-verificador-qa</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>2.4, 2.5, 2.6, 2.7, 2.8, 2.9, 2.10, 3.5, 3.6, 3.7, 3.8, 5.4, 6.1, 6.5, 6.8, 6.9; P-15, P-20, P-22 a P-35, P-43 a P-47</t>
+          <t>6.3, 2.11; P-39, P-48, P-49, P-50</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Botones de /, /ingresar, /ingresar/codigo, /afiliacion, /afiliacion/enviada y /cuenta funcionando en local</t>
+          <t>QA 1 de punta a punta: 186 pruebas pasan, 2 fallan</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Hecho: 2.5–2.10 y 3.5–3.7 (ingreso con código, proxy, Salir, Mis datos, afiliación con límites y honeypot, crédito conectado a /cuenta), contra Supabase local. En curso: 2.4 (plantilla local con {{ .Token }} lista; faltan SMTP y plantilla en producción), 3.8 (correos con Resend listos, falta RESEND_API_KEY), 5.4 (placeholder de /politica-de-datos, falta el texto de la cooperativa), 6.1 (pruebas de zod y /cuenta; faltan las de Server Actions). Dependencias: se quitó 2.4 de 2.5 y 2.9 porque el código funciona en local sin la configuración de producción; en su lugar 6.5 (despliegue) pasa a depender de 2.4, y 6.6/6.7 lo heredan vía 6.5. 3.8 y 4.3 siguen dependiendo de 2.4. Nuevas: 6.8 migración 20260923210000_limite_de_intentos.sql en producción (peso 1) y 6.9 variables en Vercel (peso 1), ambas antes de 6.5. Pendientes nuevos: P-43 (migración), P-44 (Vercel), P-45 (vencimiento 10 min e intervalo ≤ 45 s en Supabase, ligado a 2.4), P-46 (nombres de grados) y P-47 (estado de desembolso) de la cooperativa; 5.3 suma estos dos datos a su bloqueo.</t>
+          <t>Playwright contra Supabase local (1280 y 390 px); pruebas en tests/e2e/ e informe en docs/verificaciones/2026-09-23-verificacion-1.md. Sin fallas críticas ni altas; una media (F-01: el select «Grado» de /afiliacion se vacía tras un error de validación). 6.3 y P-39 pasan a En curso (falta ga-verificador-responsive). Nueva actividad 2.11 (corregir F-01, peso 1, depende de 2.9) y 6.3 pasa a depender de ella. Pendientes nuevos: P-48 (F-01), P-49 (revisar x-forwarded-for para el límite por IP, ligado a 6.2) y P-50 (confirmar el envío de los correos de afiliación, ligado a 3.8).</t>
         </is>
       </c>
     </row>
@@ -36837,20 +37194,47 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
+          <t>ga-funcionalidad-botones</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>2.4, 2.5, 2.6, 2.7, 2.8, 2.9, 2.10, 3.5, 3.6, 3.7, 3.8, 5.4, 6.1, 6.5, 6.8, 6.9; P-15, P-20, P-22 a P-35, P-43 a P-47</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Botones de /, /ingresar, /ingresar/codigo, /afiliacion, /afiliacion/enviada y /cuenta funcionando en local</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Hecho: 2.5–2.10 y 3.5–3.7 (ingreso con código, proxy, Salir, Mis datos, afiliación con límites y honeypot, crédito conectado a /cuenta), contra Supabase local. En curso: 2.4 (plantilla local con {{ .Token }} lista; faltan SMTP y plantilla en producción), 3.8 (correos con Resend listos, falta RESEND_API_KEY), 5.4 (placeholder de /politica-de-datos, falta el texto de la cooperativa), 6.1 (pruebas de zod y /cuenta; faltan las de Server Actions). Dependencias: se quitó 2.4 de 2.5 y 2.9 porque el código funciona en local sin la configuración de producción; en su lugar 6.5 (despliegue) pasa a depender de 2.4, y 6.6/6.7 lo heredan vía 6.5. 3.8 y 4.3 siguen dependiendo de 2.4. Nuevas: 6.8 migración 20260923210000_limite_de_intentos.sql en producción (peso 1) y 6.9 variables en Vercel (peso 1), ambas antes de 6.5. Pendientes nuevos: P-43 (migración), P-44 (Vercel), P-45 (vencimiento 10 min e intervalo ≤ 45 s en Supabase, ligado a 2.4), P-46 (nombres de grados) y P-47 (estado de desembolso) de la cooperativa; 5.3 suma estos dos datos a su bloqueo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
           <t>Claude (sesión principal)</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Todas</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Creación del Excel de avances</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>Pendientes desde PENDIENTES.md, plan desde la propuesta (6 fases, 8 semanas) reorganizado en 2 filas con cola infinita y pesos 1–5.</t>
         </is>

</xml_diff>